<commit_message>
Format đề DELF: A1 đối chiếu sujet d'exemple chính thức (CO 5 bài 4/4/4/8/5, CE 6/6/6/7, PE 10+15)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/format-de-thi-DELF-A1-B2.xlsx
+++ b/docs/format-de-thi-DELF-A1-B2.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="237">
   <si>
     <t>Trình độ</t>
   </si>
@@ -77,18 +77,21 @@
     <t>≥ 50/100 và mỗi kỹ năng ≥ 5/25</t>
   </si>
   <si>
+    <t>Chính thức (sujet d'exemple A1, delfdalf.ch)</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>1 giờ 40</t>
+  </si>
+  <si>
+    <t>6 đến 8 phút</t>
+  </si>
+  <si>
     <t>Thứ cấp (tài liệu luyện thi), cần đối chiếu sujet mẫu FEI</t>
   </si>
   <si>
-    <t>A2</t>
-  </si>
-  <si>
-    <t>1 giờ 40</t>
-  </si>
-  <si>
-    <t>6 đến 8 phút</t>
-  </si>
-  <si>
     <t>B1</t>
   </si>
   <si>
@@ -149,159 +152,210 @@
     <t>CO</t>
   </si>
   <si>
-    <t>Hiểu thông báo, tin nhắn ngắn đời sống hằng ngày</t>
-  </si>
-  <si>
-    <t>Thông báo, tin nhắn thoại</t>
-  </si>
-  <si>
-    <t>3 đến 4 tài liệu rất ngắn cho cả phần</t>
+    <t>Hiểu tin nhắn trên máy trả lời</t>
+  </si>
+  <si>
+    <t>Tin nhắn thoại</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
   <si>
     <t>2 lần</t>
   </si>
   <si>
-    <t>QCM (A/B/C), có thể chọn hình</t>
-  </si>
-  <si>
-    <t>Tổng audio rất ngắn, tối đa khoảng 3 phút</t>
-  </si>
-  <si>
-    <t>Hiểu tin nhắn thoại</t>
-  </si>
-  <si>
-    <t>Tin nhắn trên máy trả lời</t>
+    <t>QCM (chọn hình hoặc chữ)</t>
+  </si>
+  <si>
+    <t>4 điểm</t>
+  </si>
+  <si>
+    <t>Chính thức (sujet d'exemple A1 tout public, delfdalf.ch 2022)</t>
+  </si>
+  <si>
+    <t>Hiểu thông báo</t>
+  </si>
+  <si>
+    <t>Thông báo nơi công cộng</t>
+  </si>
+  <si>
+    <t>QCM</t>
+  </si>
+  <si>
+    <t>Hiểu tin nhắn / thông báo ngắn</t>
+  </si>
+  <si>
+    <t>Tin nhắn</t>
+  </si>
+  <si>
+    <t>Nhận diện tình huống của 4 hội thoại ngắn</t>
+  </si>
+  <si>
+    <t>4 hội thoại, nghỉ 15 giây sau mỗi hội thoại</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Ghép hội thoại với 6 HÌNH (A–F)</t>
+  </si>
+  <si>
+    <t>8 điểm (2 điểm mỗi hội thoại)</t>
+  </si>
+  <si>
+    <t>Nhận ra đồ vật được nhắc trong một tin nhắn</t>
+  </si>
+  <si>
+    <t>Có / Không cho 5 đồ vật (có hình)</t>
+  </si>
+  <si>
+    <t>5 điểm</t>
+  </si>
+  <si>
+    <t>CE</t>
+  </si>
+  <si>
+    <t>Đọc tin nhắn của một người bạn</t>
+  </si>
+  <si>
+    <t>Tin nhắn / email</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>QCM</t>
-  </si>
-  <si>
-    <t>Hiểu thông báo nơi công cộng / radio ngắn</t>
+    <t>QCM + trả lời ngắn</t>
+  </si>
+  <si>
+    <t>6 điểm</t>
+  </si>
+  <si>
+    <t>Đọc chỉ dẫn đường đi</t>
+  </si>
+  <si>
+    <t>Tài liệu kèm sơ đồ</t>
+  </si>
+  <si>
+    <t>QCM (có hình)</t>
+  </si>
+  <si>
+    <t>Đọc thời gian biểu / lịch hoạt động</t>
+  </si>
+  <si>
+    <t>Lịch, bảng giờ</t>
+  </si>
+  <si>
+    <t>Đọc quảng cáo / tờ thông tin</t>
+  </si>
+  <si>
+    <t>Tờ quảng cáo</t>
+  </si>
+  <si>
+    <t>7 điểm</t>
+  </si>
+  <si>
+    <t>PE</t>
+  </si>
+  <si>
+    <t>Điền phiếu (ví dụ phiếu khách sạn)</t>
+  </si>
+  <si>
+    <t>Phiếu 10 ô: ngày sinh, quốc tịch, email, địa chỉ, mã bưu chính, nước, điện thoại, nghề, ngày</t>
+  </si>
+  <si>
+    <t>Điền thông tin</t>
+  </si>
+  <si>
+    <t>10 điểm, 1 điểm mỗi ô</t>
+  </si>
+  <si>
+    <t>Viết thư/tin nhắn cho bạn (mời, kể hoạt động)</t>
+  </si>
+  <si>
+    <t>Thư thân mật</t>
+  </si>
+  <si>
+    <t>Tự luận</t>
+  </si>
+  <si>
+    <t>15 điểm, tối thiểu 40 từ</t>
+  </si>
+  <si>
+    <t>PO</t>
+  </si>
+  <si>
+    <t>Entretien dirigé (trả lời câu hỏi về bản thân)</t>
+  </si>
+  <si>
+    <t>Không chuẩn bị</t>
+  </si>
+  <si>
+    <t>Khoảng 1 phút</t>
+  </si>
+  <si>
+    <t>Échange d'informations (hỏi từ thẻ gợi ý)</t>
+  </si>
+  <si>
+    <t>Khoảng 2 phút</t>
+  </si>
+  <si>
+    <t>Dialogue simulé (mua bán, đặt hàng)</t>
+  </si>
+  <si>
+    <t>Có 10 phút chuẩn bị cho phần 2 và 3</t>
+  </si>
+  <si>
+    <t>Hiểu thông báo nơi công cộng</t>
   </si>
   <si>
     <t>Thông báo</t>
   </si>
   <si>
+    <t>Cả phần khoảng 14 tài liệu ngắn, khoảng 20 câu</t>
+  </si>
+  <si>
+    <t>QCM (A/B/C)</t>
+  </si>
+  <si>
+    <t>Tài liệu tối đa khoảng 5 phút; format mới bỏ câu điền</t>
+  </si>
+  <si>
+    <t>Hiểu tin nhắn thoại / radio</t>
+  </si>
+  <si>
+    <t>Tin nhắn, bản tin ngắn</t>
+  </si>
+  <si>
+    <t>Hiểu thông tin radio / phỏng vấn ngắn</t>
+  </si>
+  <si>
+    <t>Radio</t>
+  </si>
+  <si>
     <t>Nhận diện tình huống hội thoại</t>
   </si>
   <si>
-    <t>Đoạn hội thoại ngắn</t>
-  </si>
-  <si>
-    <t>Ghép hội thoại với tình huống/hình</t>
-  </si>
-  <si>
-    <t>CE</t>
+    <t>4 đoạn hội thoại</t>
+  </si>
+  <si>
+    <t>6 tình huống cho 4 hội thoại</t>
+  </si>
+  <si>
+    <t>Ghép hội thoại với tình huống</t>
   </si>
   <si>
     <t>1 đến 4</t>
   </si>
   <si>
-    <t>Đọc tài liệu đời sống: tin nhắn, thư ngắn, quảng cáo, thời gian biểu, chỉ dẫn</t>
-  </si>
-  <si>
-    <t>Tài liệu thực tế rất ngắn</t>
+    <t>Đọc tài liệu đời sống: thư, email, quảng cáo, chỉ dẫn, bài báo ngắn</t>
+  </si>
+  <si>
+    <t>Tài liệu thực tế</t>
   </si>
   <si>
     <t>1 tài liệu mỗi bài</t>
   </si>
   <si>
-    <t>QCM, chọn hình</t>
-  </si>
-  <si>
-    <t>Câu hỏi theo thứ tự tài liệu</t>
-  </si>
-  <si>
-    <t>PE</t>
-  </si>
-  <si>
-    <t>Điền phiếu / mẫu đơn</t>
-  </si>
-  <si>
-    <t>Phiếu thông tin</t>
-  </si>
-  <si>
-    <t>Điền thông tin cá nhân</t>
-  </si>
-  <si>
-    <t>Viết tin nhắn, bưu thiếp, thư ngắn</t>
-  </si>
-  <si>
-    <t>Câu đơn giản về đời sống</t>
-  </si>
-  <si>
-    <t>Tự luận</t>
-  </si>
-  <si>
-    <t>Tối thiểu 40 từ</t>
-  </si>
-  <si>
-    <t>PO</t>
-  </si>
-  <si>
-    <t>Entretien dirigé (trả lời câu hỏi về bản thân)</t>
-  </si>
-  <si>
-    <t>Không chuẩn bị</t>
-  </si>
-  <si>
-    <t>Khoảng 1 phút</t>
-  </si>
-  <si>
-    <t>Échange d'informations (hỏi từ thẻ gợi ý)</t>
-  </si>
-  <si>
-    <t>Khoảng 2 phút</t>
-  </si>
-  <si>
-    <t>Dialogue simulé (mua bán, đặt hàng)</t>
-  </si>
-  <si>
-    <t>Có 10 phút chuẩn bị cho phần 2 và 3</t>
-  </si>
-  <si>
-    <t>Hiểu thông báo nơi công cộng</t>
-  </si>
-  <si>
-    <t>Cả phần khoảng 14 tài liệu ngắn, khoảng 20 câu</t>
-  </si>
-  <si>
-    <t>QCM (A/B/C)</t>
-  </si>
-  <si>
-    <t>Tài liệu tối đa khoảng 5 phút; format mới bỏ câu điền</t>
-  </si>
-  <si>
-    <t>Hiểu tin nhắn thoại / radio</t>
-  </si>
-  <si>
-    <t>Tin nhắn, bản tin ngắn</t>
-  </si>
-  <si>
-    <t>Hiểu thông tin radio / phỏng vấn ngắn</t>
-  </si>
-  <si>
-    <t>Radio</t>
-  </si>
-  <si>
-    <t>4 đoạn hội thoại</t>
-  </si>
-  <si>
-    <t>6 tình huống cho 4 hội thoại</t>
-  </si>
-  <si>
-    <t>Ghép hội thoại với tình huống</t>
-  </si>
-  <si>
-    <t>Đọc tài liệu đời sống: thư, email, quảng cáo, chỉ dẫn, bài báo ngắn</t>
-  </si>
-  <si>
-    <t>Tài liệu thực tế</t>
-  </si>
-  <si>
     <t>QCM (format mới)</t>
   </si>
   <si>
@@ -317,9 +371,6 @@
     <t>Viết thư/tin nhắn: mời, cảm ơn, xin lỗi, yêu cầu, thông báo</t>
   </si>
   <si>
-    <t>Thư thân mật</t>
-  </si>
-  <si>
     <t>Entretien dirigé</t>
   </si>
   <si>
@@ -347,9 +398,6 @@
     <t>Hội thoại</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>Theo đề</t>
   </si>
   <si>
@@ -554,39 +602,42 @@
     <t>Ghi chú khi soạn</t>
   </si>
   <si>
-    <t>Khoảng 15 đến 20 câu QCM</t>
-  </si>
-  <si>
-    <t>Audio rất ngắn, mỗi bài nghe 2 lần. Không dùng câu điền.</t>
+    <t>4 + 4 + 4 + 8 + 5 điểm</t>
+  </si>
+  <si>
+    <t>Bài 4 ghép 4 hội thoại với 6 hình (nghỉ 15 giây sau mỗi hội thoại); bài 5 Có/Không cho 5 đồ vật. Mỗi bài nghe 2 lần, tổng audio tối đa 3 phút.</t>
+  </si>
+  <si>
+    <t>6 + 6 + 6 + 7 điểm</t>
+  </si>
+  <si>
+    <t>Tài liệu đời sống thật, nhiều câu chọn hình.</t>
+  </si>
+  <si>
+    <t>Phiếu 10 điểm + thư 15 điểm</t>
+  </si>
+  <si>
+    <t>Phiếu 10 ô, 1 điểm mỗi ô; thư ≥ 40 từ.</t>
+  </si>
+  <si>
+    <t>Không chấm</t>
+  </si>
+  <si>
+    <t>1 đến 3</t>
+  </si>
+  <si>
+    <t>App chỉ ghi âm, không chấm điểm phần nói.</t>
+  </si>
+  <si>
+    <t>Khoảng 20 câu QCM</t>
+  </si>
+  <si>
+    <t>Khoảng 14 tài liệu ngắn; bài 4 ghép 4 hội thoại với 6 tình huống.</t>
   </si>
   <si>
     <t>Khoảng 15 đến 20 câu</t>
   </si>
   <si>
-    <t>Tài liệu đời sống thật, có thể dùng hình.</t>
-  </si>
-  <si>
-    <t>1 phiếu + 1 câu tự luận</t>
-  </si>
-  <si>
-    <t>Câu tự luận yêu cầu ≥ 40 từ.</t>
-  </si>
-  <si>
-    <t>Không chấm</t>
-  </si>
-  <si>
-    <t>1 đến 3</t>
-  </si>
-  <si>
-    <t>App chỉ ghi âm, không chấm điểm phần nói.</t>
-  </si>
-  <si>
-    <t>Khoảng 20 câu QCM</t>
-  </si>
-  <si>
-    <t>Khoảng 14 tài liệu ngắn; bài 4 ghép 4 hội thoại với 6 tình huống.</t>
-  </si>
-  <si>
     <t>2 câu tự luận</t>
   </si>
   <si>
@@ -665,10 +716,16 @@
     <t>delfdalf.jp/diplomes-et-tests/delf-tout-public; digischool.fr (format QCM); getsetfrench.com, communfrancais.com (cải cách 2020). Trang FEI chặn truy cập tự động nên chưa đọc được bản gốc A1/A2.</t>
   </si>
   <si>
+    <t>Đã đối chiếu A1 (08/10)</t>
+  </si>
+  <si>
+    <t>Sujet d'exemple A1 tout public (delfdalf.ch, 2022): CO 5 bài 4/4/4/8/5 điểm, CE 4 bài 6/6/6/7, PE phiếu 10 + thư 15. Đề FRACILE A1 · Đề 1 hiện có 4 bài nghe: THIẾU bài 5 (Có/Không) và bài 4 dùng chữ thay hình.</t>
+  </si>
+  <si>
     <t>Việc nên làm tiếp</t>
   </si>
   <si>
-    <t>Tải sujet-démo A1, A2 chính thức trên france-education-international.fr để xác nhận số câu và điểm từng bài trước khi soạn đề hàng loạt.</t>
+    <t>A2: chưa tải được sujet d'exemple (đường dẫn delfdalf.ch trả 404). Thêm bài nghe 5 cho đề A1.</t>
   </si>
 </sst>
 </file>
@@ -1195,7 +1252,7 @@
         <v>17</v>
       </c>
       <c r="H2" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I2" s="4">
         <v>4</v>
@@ -1257,12 +1314,12 @@
         <v>19</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="4">
         <v>25</v>
@@ -1274,19 +1331,19 @@
         <v>45</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H4" s="4">
         <v>3</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J4" s="4">
         <v>1</v>
@@ -1301,12 +1358,12 @@
         <v>19</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B5" s="4">
         <v>30</v>
@@ -1318,19 +1375,19 @@
         <v>60</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J5" s="4">
         <v>1</v>
@@ -1345,7 +1402,7 @@
         <v>19</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1357,7 +1414,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -1375,28 +1432,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>13</v>
@@ -1407,31 +1464,31 @@
         <v>14</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1439,31 +1496,31 @@
         <v>14</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C3" s="4">
         <v>2</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="I3" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="J3" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1471,31 +1528,31 @@
         <v>14</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C4" s="4">
         <v>3</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>53</v>
-      </c>
       <c r="I4" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1503,31 +1560,31 @@
         <v>14</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C5" s="4">
         <v>4</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1535,31 +1592,31 @@
         <v>14</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>60</v>
+        <v>44</v>
+      </c>
+      <c r="C6" s="4">
+        <v>5</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="F6" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="G6" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H6" s="4" t="s">
+      <c r="I6" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="I6" s="4" t="s">
-        <v>65</v>
-      </c>
       <c r="J6" s="4" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1567,31 +1624,31 @@
         <v>14</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C7" s="4">
         <v>1</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>68</v>
-      </c>
       <c r="F7" s="4" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>69</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1599,31 +1656,31 @@
         <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C8" s="4">
         <v>2</v>
       </c>
       <c r="D8" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I8" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>73</v>
-      </c>
       <c r="J8" s="4" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1631,31 +1688,31 @@
         <v>14</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="4">
+        <v>3</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C9" s="4">
-        <v>1</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>52</v>
-      </c>
       <c r="F9" s="4" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1663,31 +1720,31 @@
         <v>14</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="C10" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D10" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I10" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>79</v>
-      </c>
       <c r="J10" s="4" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1695,159 +1752,159 @@
         <v>14</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C11" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>80</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>52</v>
+        <v>81</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I11" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="J11" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>43</v>
-      </c>
       <c r="C12" s="4">
+        <v>2</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C13" s="4">
         <v>1</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" s="4">
+      <c r="D13" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C14" s="4">
         <v>2</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="4">
+      <c r="D14" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C15" s="4">
         <v>3</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" s="4">
-        <v>4</v>
-      </c>
       <c r="D15" s="4" t="s">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>52</v>
+        <v>93</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1855,31 +1912,31 @@
         <v>21</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>60</v>
+        <v>44</v>
+      </c>
+      <c r="C16" s="4">
+        <v>1</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>63</v>
+        <v>98</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>52</v>
+        <v>100</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1887,31 +1944,31 @@
         <v>21</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="C17" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1919,31 +1976,31 @@
         <v>21</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="C18" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1951,31 +2008,31 @@
         <v>21</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>74</v>
+        <v>44</v>
       </c>
       <c r="C19" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>52</v>
+        <v>106</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>52</v>
+        <v>107</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>102</v>
+        <v>68</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1983,31 +2040,31 @@
         <v>21</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C20" s="4">
-        <v>2</v>
+        <v>65</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>109</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>52</v>
+        <v>111</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>52</v>
+        <v>112</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2015,575 +2072,703 @@
         <v>21</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C21" s="4">
+        <v>1</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" s="4">
+        <v>2</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" s="4">
+        <v>1</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C24" s="4">
+        <v>2</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C25" s="4">
         <v>3</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="J21" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
+      <c r="D25" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="J25" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="4">
-        <v>1</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="J22" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="4">
-        <v>2</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="I23" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="J23" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="4">
-        <v>3</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="J24" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C25" s="4">
-        <v>1</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H25" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="I25" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="J25" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>121</v>
+        <v>44</v>
+      </c>
+      <c r="C26" s="4">
+        <v>1</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>124</v>
+        <v>47</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>52</v>
+        <v>127</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="C27" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G27" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="E27" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>52</v>
-      </c>
       <c r="H27" s="4" t="s">
-        <v>129</v>
+        <v>54</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>130</v>
+        <v>68</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>74</v>
+        <v>44</v>
       </c>
       <c r="C28" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>52</v>
+        <v>104</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>52</v>
+        <v>127</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>76</v>
+        <v>54</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>131</v>
+        <v>68</v>
       </c>
       <c r="J28" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="C29" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>132</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>52</v>
+        <v>133</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>52</v>
+        <v>134</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>76</v>
+        <v>135</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C30" s="4">
-        <v>3</v>
+        <v>65</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>17</v>
+        <v>142</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
-        <v>30</v>
+      <c r="A31" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>43</v>
+        <v>79</v>
       </c>
       <c r="C31" s="4">
         <v>1</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>110</v>
+        <v>68</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>53</v>
+        <v>145</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="7" t="s">
-        <v>30</v>
+      <c r="A32" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>43</v>
+        <v>88</v>
       </c>
       <c r="C32" s="4">
+        <v>1</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="J32" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C33" s="4">
         <v>2</v>
       </c>
-      <c r="D32" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="F32" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G32" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="H32" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="I32" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="J32" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C33" s="4">
+      <c r="D33" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="J33" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C34" s="4">
         <v>3</v>
       </c>
-      <c r="D33" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="G33" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="H33" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="I33" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="J33" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>148</v>
-      </c>
       <c r="D34" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>123</v>
+        <v>151</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>124</v>
+        <v>152</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>125</v>
+        <v>153</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>150</v>
+        <v>17</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="C35" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>110</v>
+        <v>47</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>52</v>
+        <v>156</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="C36" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>52</v>
+        <v>159</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>129</v>
+        <v>54</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>155</v>
+        <v>68</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>74</v>
+        <v>44</v>
       </c>
       <c r="C37" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>136</v>
+        <v>162</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>52</v>
+        <v>163</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>158</v>
+        <v>54</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C38" s="4">
+        <v>65</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="J38" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="4">
+        <v>3</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J39" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C40" s="4">
+        <v>1</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="J40" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C41" s="4">
+        <v>1</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J41" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C42" s="4">
         <v>2</v>
       </c>
-      <c r="D38" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G38" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H38" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="I38" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="J38" s="4" t="s">
-        <v>29</v>
+      <c r="D42" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="J42" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -2608,7 +2793,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>11</v>
@@ -2619,226 +2804,226 @@
     </row>
     <row r="2" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="C2" s="4">
         <v>2</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="C3" s="4">
         <v>4</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="C4" s="4">
         <v>4</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="C5" s="4">
         <v>3</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="C6" s="4">
         <v>6</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="C7" s="4">
         <v>6</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="C8" s="4">
         <v>25</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="C9" s="4">
         <v>2</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="C10" s="4">
         <v>2</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="C11" s="4">
         <v>3</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="C12" s="4">
         <v>3</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="C13" s="4">
         <v>4</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="C14" s="4">
         <v>5</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="C15" s="4">
         <v>6</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="C16" s="4">
         <v>25</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>172</v>
+        <v>188</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -2864,22 +3049,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>178</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2887,7 +3072,7 @@
         <v>14</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C2" s="4">
         <v>20</v>
@@ -2896,13 +3081,13 @@
         <v>25</v>
       </c>
       <c r="E2" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>179</v>
+        <v>195</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>180</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2910,7 +3095,7 @@
         <v>14</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C3" s="4">
         <v>30</v>
@@ -2922,10 +3107,10 @@
         <v>4</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>181</v>
+        <v>197</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2933,7 +3118,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C4" s="4">
         <v>30</v>
@@ -2945,10 +3130,10 @@
         <v>2</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2956,22 +3141,22 @@
         <v>14</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="C5" s="4">
         <v>10</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2979,7 +3164,7 @@
         <v>21</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C6" s="4">
         <v>25</v>
@@ -2991,10 +3176,10 @@
         <v>4</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>188</v>
+        <v>204</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>189</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3002,7 +3187,7 @@
         <v>21</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C7" s="4">
         <v>30</v>
@@ -3014,10 +3199,10 @@
         <v>4</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>181</v>
+        <v>206</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3025,7 +3210,7 @@
         <v>21</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C8" s="4">
         <v>45</v>
@@ -3037,10 +3222,10 @@
         <v>2</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>190</v>
+        <v>207</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>191</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3048,30 +3233,30 @@
         <v>21</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="C9" s="4">
         <v>12</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C10" s="4">
         <v>25</v>
@@ -3083,18 +3268,18 @@
         <v>3</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>192</v>
+        <v>209</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C11" s="4">
         <v>45</v>
@@ -3103,21 +3288,21 @@
         <v>25</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>195</v>
+        <v>212</v>
       </c>
     </row>
     <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C12" s="4">
         <v>45</v>
@@ -3129,41 +3314,41 @@
         <v>1</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>196</v>
+        <v>213</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="C13" s="4">
         <v>15</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C14" s="4">
         <v>30</v>
@@ -3172,21 +3357,21 @@
         <v>25</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C15" s="4">
         <v>60</v>
@@ -3195,21 +3380,21 @@
         <v>25</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>199</v>
+        <v>216</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="C16" s="4">
         <v>60</v>
@@ -3221,33 +3406,33 @@
         <v>1</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>196</v>
+        <v>213</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="C17" s="4">
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -3259,7 +3444,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" style="8" customWidth="1"/>
@@ -3268,66 +3453,74 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>202</v>
+        <v>219</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>203</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>204</v>
+        <v>221</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>205</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>206</v>
+        <v>223</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>207</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>209</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>210</v>
+        <v>227</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>212</v>
+        <v>229</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>213</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>215</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>216</v>
+        <v>233</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>217</v>
+        <v>234</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>